<commit_message>
Change subject B to "we built" for consistency with the body's voice
The body opens "We built it because..." in first-person plural even though
Austin writes as an individual founder throughout; subject B had drifted to
"I built" instead. Austin caught the mismatch. Updated the locked contract
and regenerated the final spreadsheet, keeping all 67 verified addresses,
statuses and the A/B split intact.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ks9xKVaecPLqBHjpvz4BFJ
</commit_message>
<xml_diff>
--- a/.claude/skills/outreach-drafting/state/drafts/healthcare-outreach-verified-2026-09-02.xlsx
+++ b/.claude/skills/outreach-drafting/state/drafts/healthcare-outreach-verified-2026-09-02.xlsx
@@ -454,7 +454,7 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
@@ -541,10 +541,15 @@
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Barbara,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Tue Sept 8 at 9:30 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Tue Sept 8 at 9:30 ET?
 Austin</t>
         </is>
       </c>
@@ -583,16 +588,21 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Kim,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Wed Sept 9 at 10:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Wed Sept 9 at 10:00 ET?
 Austin</t>
         </is>
       </c>
@@ -637,10 +647,15 @@
       <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Kat,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Thu Sept 10 at 10:30 CT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Thu Sept 10 at 10:30 CT?
 Austin</t>
         </is>
       </c>
@@ -679,16 +694,21 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Sara,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Fri Sept 11 at 11:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Fri Sept 11 at 11:00 ET?
 Austin</t>
         </is>
       </c>
@@ -733,10 +753,15 @@
       <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Shantel,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Tue Sept 8 at 1:30 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Tue Sept 8 at 1:30 ET?
 Austin</t>
         </is>
       </c>
@@ -775,16 +800,21 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Cris,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Wed Sept 9 at 2:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Wed Sept 9 at 2:00 ET?
 Austin</t>
         </is>
       </c>
@@ -829,10 +859,15 @@
       <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Valerie,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Thu Sept 10 at 2:30 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Thu Sept 10 at 2:30 ET?
 Austin</t>
         </is>
       </c>
@@ -867,16 +902,21 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Amber,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Fri Sept 11 at 3:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Fri Sept 11 at 3:00 ET?
 Austin</t>
         </is>
       </c>
@@ -921,10 +961,15 @@
       <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Jeanne,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Tue Sept 8 at 9:30 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Tue Sept 8 at 9:30 ET?
 Austin</t>
         </is>
       </c>
@@ -963,16 +1008,21 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Melanie,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Wed Sept 9 at 10:00 PT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Wed Sept 9 at 10:00 PT?
 Austin</t>
         </is>
       </c>
@@ -1017,10 +1067,15 @@
       <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Jennifer,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Thu Sept 10 at 10:30 MT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Thu Sept 10 at 10:30 MT?
 Austin</t>
         </is>
       </c>
@@ -1059,16 +1114,21 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Hollie,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Fri Sept 11 at 11:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Fri Sept 11 at 11:00 ET?
 Austin</t>
         </is>
       </c>
@@ -1113,10 +1173,15 @@
       <c r="G14" s="4" t="inlineStr">
         <is>
           <t>David,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Tue Sept 8 at 1:30 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Tue Sept 8 at 1:30 ET?
 Austin</t>
         </is>
       </c>
@@ -1155,16 +1220,21 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Colton,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Wed Sept 9 at 2:00 MT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Wed Sept 9 at 2:00 MT?
 Austin</t>
         </is>
       </c>
@@ -1209,10 +1279,15 @@
       <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Michael,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Thu Sept 10 at 2:30 MT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Thu Sept 10 at 2:30 MT?
 Austin</t>
         </is>
       </c>
@@ -1251,16 +1326,21 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Paul,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Fri Sept 11 at 3:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Fri Sept 11 at 3:00 ET?
 Austin</t>
         </is>
       </c>
@@ -1305,10 +1385,15 @@
       <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Cheryl,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Tue Sept 8 at 9:30 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Tue Sept 8 at 9:30 ET?
 Austin</t>
         </is>
       </c>
@@ -1347,16 +1432,21 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Donnie,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Wed Sept 9 at 10:00 CT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Wed Sept 9 at 10:00 CT?
 Austin</t>
         </is>
       </c>
@@ -1401,10 +1491,15 @@
       <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Keith,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Thu Sept 10 at 10:30 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Thu Sept 10 at 10:30 ET?
 Austin</t>
         </is>
       </c>
@@ -1443,16 +1538,21 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Barbara,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Fri Sept 11 at 11:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Fri Sept 11 at 11:00 ET?
 Austin</t>
         </is>
       </c>
@@ -1497,10 +1597,15 @@
       <c r="G22" s="2" t="inlineStr">
         <is>
           <t>Suzette,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Tue Sept 8 at 1:30 PT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Tue Sept 8 at 1:30 PT?
 Austin</t>
         </is>
       </c>
@@ -1539,16 +1644,21 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Danielle,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Wed Sept 9 at 2:00 MT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Wed Sept 9 at 2:00 MT?
 Austin</t>
         </is>
       </c>
@@ -1593,10 +1703,15 @@
       <c r="G24" s="3" t="inlineStr">
         <is>
           <t>Melissa,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Thu Sept 10 at 2:30 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Thu Sept 10 at 2:30 ET?
 Austin</t>
         </is>
       </c>
@@ -1635,16 +1750,21 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
           <t>Michael,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Fri Sept 11 at 3:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Fri Sept 11 at 3:00 ET?
 Austin</t>
         </is>
       </c>
@@ -1689,10 +1809,15 @@
       <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Suzann,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Tue Sept 8 at 9:30 CT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Tue Sept 8 at 9:30 CT?
 Austin</t>
         </is>
       </c>
@@ -1727,16 +1852,21 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Jamie,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Wed Sept 9 at 10:00 CT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Wed Sept 9 at 10:00 CT?
 Austin</t>
         </is>
       </c>
@@ -1781,10 +1911,15 @@
       <c r="G28" s="3" t="inlineStr">
         <is>
           <t>Meredith,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Thu Sept 10 at 10:30 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Thu Sept 10 at 10:30 ET?
 Austin</t>
         </is>
       </c>
@@ -1823,16 +1958,21 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
           <t>Bill,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Fri Sept 11 at 11:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Fri Sept 11 at 11:00 ET?
 Austin</t>
         </is>
       </c>
@@ -1877,10 +2017,15 @@
       <c r="G30" s="3" t="inlineStr">
         <is>
           <t>Maria,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Tue Sept 8 at 1:30 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Tue Sept 8 at 1:30 ET?
 Austin</t>
         </is>
       </c>
@@ -1919,16 +2064,21 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
           <t>Nicole,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Wed Sept 9 at 2:00 CT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Wed Sept 9 at 2:00 CT?
 Austin</t>
         </is>
       </c>
@@ -1973,10 +2123,15 @@
       <c r="G32" s="2" t="inlineStr">
         <is>
           <t>Christina,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Thu Sept 10 at 2:30 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Thu Sept 10 at 2:30 ET?
 Austin</t>
         </is>
       </c>
@@ -2015,16 +2170,21 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
           <t>Jeannene,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Fri Sept 11 at 3:00 PT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Fri Sept 11 at 3:00 PT?
 Austin</t>
         </is>
       </c>
@@ -2069,10 +2229,15 @@
       <c r="G34" s="4" t="inlineStr">
         <is>
           <t>Kimberly,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Tue Sept 8 at 9:30 PT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Tue Sept 8 at 9:30 PT?
 Austin</t>
         </is>
       </c>
@@ -2107,16 +2272,21 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Ann,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Wed Sept 9 at 10:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Wed Sept 9 at 10:00 ET?
 Austin</t>
         </is>
       </c>
@@ -2157,10 +2327,15 @@
       <c r="G36" s="3" t="inlineStr">
         <is>
           <t>Sandra,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Thu Sept 10 at 10:30 PT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Thu Sept 10 at 10:30 PT?
 Austin</t>
         </is>
       </c>
@@ -2199,16 +2374,21 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
           <t>Erin,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Fri Sept 11 at 11:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Fri Sept 11 at 11:00 ET?
 Austin</t>
         </is>
       </c>
@@ -2253,10 +2433,15 @@
       <c r="G38" s="3" t="inlineStr">
         <is>
           <t>Michelle,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Tue Sept 8 at 1:30 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Tue Sept 8 at 1:30 ET?
 Austin</t>
         </is>
       </c>
@@ -2295,16 +2480,21 @@
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G39" s="4" t="inlineStr">
         <is>
           <t>Zoe,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Wed Sept 9 at 2:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Wed Sept 9 at 2:00 ET?
 Austin</t>
         </is>
       </c>
@@ -2349,10 +2539,15 @@
       <c r="G40" s="4" t="inlineStr">
         <is>
           <t>Vamsi,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Thu Sept 10 at 2:30 CT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Thu Sept 10 at 2:30 CT?
 Austin</t>
         </is>
       </c>
@@ -2391,16 +2586,21 @@
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
           <t>Sarah,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Fri Sept 11 at 3:00 CT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Fri Sept 11 at 3:00 CT?
 Austin</t>
         </is>
       </c>
@@ -2445,10 +2645,15 @@
       <c r="G42" s="4" t="inlineStr">
         <is>
           <t>Sophia,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Tue Sept 8 at 9:30 MT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Tue Sept 8 at 9:30 MT?
 Austin</t>
         </is>
       </c>
@@ -2487,16 +2692,21 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
           <t>Ken,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Wed Sept 9 at 10:00 CT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Wed Sept 9 at 10:00 CT?
 Austin</t>
         </is>
       </c>
@@ -2541,10 +2751,15 @@
       <c r="G44" s="3" t="inlineStr">
         <is>
           <t>David,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Thu Sept 10 at 10:30 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Thu Sept 10 at 10:30 ET?
 Austin</t>
         </is>
       </c>
@@ -2583,16 +2798,21 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
           <t>Cacey,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Fri Sept 11 at 11:00 CT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Fri Sept 11 at 11:00 CT?
 Austin</t>
         </is>
       </c>
@@ -2637,10 +2857,15 @@
       <c r="G46" s="2" t="inlineStr">
         <is>
           <t>Seran,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Tue Sept 8 at 1:30 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Tue Sept 8 at 1:30 ET?
 Austin</t>
         </is>
       </c>
@@ -2679,16 +2904,21 @@
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
           <t>Rob,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Wed Sept 9 at 2:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Wed Sept 9 at 2:00 ET?
 Austin</t>
         </is>
       </c>
@@ -2733,10 +2963,15 @@
       <c r="G48" s="2" t="inlineStr">
         <is>
           <t>Holly,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Thu Sept 10 at 2:30 CT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Thu Sept 10 at 2:30 CT?
 Austin</t>
         </is>
       </c>
@@ -2775,16 +3010,21 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
           <t>Johannette,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Fri Sept 11 at 3:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Fri Sept 11 at 3:00 ET?
 Austin</t>
         </is>
       </c>
@@ -2829,10 +3069,15 @@
       <c r="G50" s="2" t="inlineStr">
         <is>
           <t>Christina,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Tue Sept 8 at 9:30 MT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Tue Sept 8 at 9:30 MT?
 Austin</t>
         </is>
       </c>
@@ -2871,16 +3116,21 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
           <t>Kaley,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Wed Sept 9 at 10:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Wed Sept 9 at 10:00 ET?
 Austin</t>
         </is>
       </c>
@@ -2921,10 +3171,15 @@
       <c r="G52" s="3" t="inlineStr">
         <is>
           <t>Joe,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Thu Sept 10 at 10:30 CT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Thu Sept 10 at 10:30 CT?
 Austin</t>
         </is>
       </c>
@@ -2963,16 +3218,21 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
           <t>Holley,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Fri Sept 11 at 11:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Fri Sept 11 at 11:00 ET?
 Austin</t>
         </is>
       </c>
@@ -3017,10 +3277,15 @@
       <c r="G54" s="3" t="inlineStr">
         <is>
           <t>Kevin,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Tue Sept 8 at 1:30 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Tue Sept 8 at 1:30 ET?
 Austin</t>
         </is>
       </c>
@@ -3059,16 +3324,21 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
           <t>Cassidy,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Wed Sept 9 at 2:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Wed Sept 9 at 2:00 ET?
 Austin</t>
         </is>
       </c>
@@ -3113,10 +3383,15 @@
       <c r="G56" s="2" t="inlineStr">
         <is>
           <t>Michelle,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Thu Sept 10 at 2:30 CT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Thu Sept 10 at 2:30 CT?
 Austin</t>
         </is>
       </c>
@@ -3155,16 +3430,21 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
           <t>Alicia,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Fri Sept 11 at 3:00 MT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Fri Sept 11 at 3:00 MT?
 Austin</t>
         </is>
       </c>
@@ -3209,10 +3489,15 @@
       <c r="G58" s="3" t="inlineStr">
         <is>
           <t>Lydia,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Tue Sept 8 at 9:30 PT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Tue Sept 8 at 9:30 PT?
 Austin</t>
         </is>
       </c>
@@ -3251,16 +3536,21 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
           <t>Patrick,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Wed Sept 9 at 10:00 CT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Wed Sept 9 at 10:00 CT?
 Austin</t>
         </is>
       </c>
@@ -3305,10 +3595,15 @@
       <c r="G60" s="2" t="inlineStr">
         <is>
           <t>David,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Thu Sept 10 at 10:30 CT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Thu Sept 10 at 10:30 CT?
 Austin</t>
         </is>
       </c>
@@ -3347,16 +3642,21 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
           <t>Gregory,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Fri Sept 11 at 11:00 CT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Fri Sept 11 at 11:00 CT?
 Austin</t>
         </is>
       </c>
@@ -3401,10 +3701,15 @@
       <c r="G62" s="2" t="inlineStr">
         <is>
           <t>Tangee,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Tue Sept 8 at 1:30 CT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Tue Sept 8 at 1:30 CT?
 Austin</t>
         </is>
       </c>
@@ -3443,16 +3748,21 @@
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
           <t>Deborah,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Wed Sept 9 at 2:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Wed Sept 9 at 2:00 ET?
 Austin</t>
         </is>
       </c>
@@ -3497,10 +3807,15 @@
       <c r="G64" s="2" t="inlineStr">
         <is>
           <t>Angela,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Thu Sept 10 at 2:30 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Thu Sept 10 at 2:30 ET?
 Austin</t>
         </is>
       </c>
@@ -3539,16 +3854,21 @@
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
           <t>Lisa,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Fri Sept 11 at 3:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Fri Sept 11 at 3:00 ET?
 Austin</t>
         </is>
       </c>
@@ -3593,10 +3913,15 @@
       <c r="G66" s="3" t="inlineStr">
         <is>
           <t>Princy,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Tue Sept 8 at 9:30 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Tue Sept 8 at 9:30 ET?
 Austin</t>
         </is>
       </c>
@@ -3635,16 +3960,21 @@
       </c>
       <c r="F67" s="4" t="inlineStr">
         <is>
-          <t>I built an affordable HIPAA compliant chat</t>
+          <t>we built an affordable HIPAA compliant chat</t>
         </is>
       </c>
       <c r="G67" s="4" t="inlineStr">
         <is>
           <t>Karen,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Wed Sept 9 at 10:00 ET?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Wed Sept 9 at 10:00 ET?
 Austin</t>
         </is>
       </c>
@@ -3689,10 +4019,15 @@
       <c r="G68" s="2" t="inlineStr">
         <is>
           <t>Tessa,
-I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big platforms weren't made for clinics needing something simple, affordable, and HIPAA compliant.
-I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
-Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA compliance, and pricing that stays affordable. Need something? Call me, not a bot.
-I'm excited to show this to you because it's exactly what I wish I had at the clinic I worked for. Do you have 15 minutes Thu Sept 10 at 10:30 CT?
+I'm Austin, co-founder of Chanty, an internal chat tool. We built it because the big
+platforms weren't made for clinics needing something simple, affordable, and HIPAA
+compliant.
+I used to work at a family-run clinic. Group texts, nobody sure who saw what, and constant
+HIPAA worry. If you're on a bigger platform, you're over-paying for complicated compliance.
+Our base plan means no complex builds or weeks-long integration, just a signed BAA, HIPAA
+compliance, and pricing that stays affordable. Need something? Call me, not a bot.
+I'm excited to show this to you because it's exactly what I wish I had at the clinic I
+worked for. Do you have 15 minutes Thu Sept 10 at 10:30 CT?
 Austin</t>
         </is>
       </c>

</xml_diff>